<commit_message>
correct rule category cvd ihd
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements_longitudinal-FRA.xlsx
+++ b/longitudinal/data_processing_elements_longitudinal-FRA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Documents\Boulot\ProPASS\FRA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CF26FC5-1C13-4F8F-AE89-E29897DBF629}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{199531C6-C37A-4433-A6FE-B5CC7FC419E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{95E6C139-84C6-42BA-8CBB-FF1D79072BFF}"/>
   </bookViews>
@@ -6801,7 +6801,7 @@
         <v>42</v>
       </c>
       <c r="W63" t="s">
-        <v>352</v>
+        <v>68</v>
       </c>
       <c r="X63" t="s">
         <v>380</v>
@@ -9128,7 +9128,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="113" spans="1:24" ht="300" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:24" ht="285" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>112</v>
       </c>
@@ -12200,7 +12200,7 @@
         <v>42</v>
       </c>
       <c r="W175" t="s">
-        <v>352</v>
+        <v>68</v>
       </c>
       <c r="X175" t="s">
         <v>380</v>
@@ -14524,7 +14524,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="225" spans="1:24" ht="300" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:24" ht="285" x14ac:dyDescent="0.25">
       <c r="A225">
         <v>112</v>
       </c>
@@ -17596,7 +17596,7 @@
         <v>42</v>
       </c>
       <c r="W287" t="s">
-        <v>352</v>
+        <v>68</v>
       </c>
       <c r="X287" t="s">
         <v>380</v>
@@ -19920,7 +19920,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="337" spans="1:24" ht="300" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:24" ht="285" x14ac:dyDescent="0.25">
       <c r="A337">
         <v>112</v>
       </c>

</xml_diff>